<commit_message>
Publish Prague_2023_WC, RioDeJaneiro_2018_WCH, Tacen_2019_WC, Tacen_2020_WC
</commit_message>
<xml_diff>
--- a/events/Tacen_2020_WC/Tacen_2020_WC_start.xlsx
+++ b/events/Tacen_2020_WC/Tacen_2020_WC_start.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W300"/>
+  <dimension ref="A1:AC291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,17 +519,47 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>Name4</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Name5</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Name6</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>ICF_ID1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>ICF_ID2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ICF_ID3</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ICF_ID4</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ICF_ID5</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ICF_ID6</t>
         </is>
       </c>
     </row>
@@ -744,7 +774,7 @@
           <t>SATKOVA Gabriela</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>68786</t>
         </is>
@@ -802,7 +832,7 @@
           <t>CORCORAN Madison</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>106163</t>
         </is>
@@ -860,7 +890,7 @@
           <t>DUSKOVA Katerina</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>51792</t>
         </is>
@@ -918,7 +948,7 @@
           <t>KUZNETSOVA Daria</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>76780</t>
         </is>
@@ -976,7 +1006,7 @@
           <t>SEPRENYI Sara Timea</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>52211</t>
         </is>
@@ -1034,7 +1064,7 @@
           <t>KRYLOVA Kseniia</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>60639</t>
         </is>
@@ -1092,7 +1122,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -1150,7 +1180,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -1208,7 +1238,7 @@
           <t>PRIGENT Romane</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>71968</t>
         </is>
@@ -1266,7 +1296,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -1324,7 +1354,7 @@
           <t>OSCHMAUTZ Antonia</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>68839</t>
         </is>
@@ -1382,7 +1412,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -1440,7 +1470,7 @@
           <t>YAZAWA Aki</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>36486</t>
         </is>
@@ -1498,7 +1528,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -1556,7 +1586,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -1614,7 +1644,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -1672,7 +1702,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -1730,7 +1760,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -1788,7 +1818,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -1846,7 +1876,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -1904,7 +1934,7 @@
           <t>FRIEDENSON Kaelin</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>87397</t>
         </is>
@@ -1962,7 +1992,7 @@
           <t>JEVTIC Milos</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>68832</t>
         </is>
@@ -2020,7 +2050,7 @@
           <t>RUDORFER Martin</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>83774</t>
         </is>
@@ -2078,7 +2108,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -2136,7 +2166,7 @@
           <t>CURTIS Samuel</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>36683</t>
         </is>
@@ -2194,7 +2224,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -2252,7 +2282,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -2310,7 +2340,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -2368,7 +2398,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -2426,7 +2456,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -2484,7 +2514,7 @@
           <t>MARX Dimitri</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>60326</t>
         </is>
@@ -2542,7 +2572,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -2600,7 +2630,7 @@
           <t>KREJCI Jakub</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>83510</t>
         </is>
@@ -2658,7 +2688,7 @@
           <t>ZIMA Tomas</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>60019</t>
         </is>
@@ -2716,7 +2746,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -2774,7 +2804,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -2832,7 +2862,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -2890,7 +2920,7 @@
           <t>DELASSUS Anatole</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>84109</t>
         </is>
@@ -2948,7 +2978,7 @@
           <t>TSVIET Igor</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>35527</t>
         </is>
@@ -3006,7 +3036,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -3064,7 +3094,7 @@
           <t>KUDER MARUSIC Vid</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>44342</t>
         </is>
@@ -3122,7 +3152,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -3180,7 +3210,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -3238,7 +3268,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -3296,7 +3326,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -3354,7 +3384,7 @@
           <t>EIGEL Pavel</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>35458</t>
         </is>
@@ -3412,7 +3442,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -3470,7 +3500,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -3528,7 +3558,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -3586,7 +3616,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -3644,7 +3674,7 @@
           <t>CORCORAN Michaela</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>106164</t>
         </is>
@@ -3702,7 +3732,7 @@
           <t>SATO Ayano</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>60374</t>
         </is>
@@ -3760,7 +3790,7 @@
           <t>KOZYREVA Anastasia</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>60640</t>
         </is>
@@ -3818,7 +3848,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -3876,7 +3906,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -3934,7 +3964,7 @@
           <t>DOBROTVORSKA Viktoriia</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>35526</t>
         </is>
@@ -3992,7 +4022,7 @@
           <t>SATKOVA Gabriela</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>68786</t>
         </is>
@@ -4050,7 +4080,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -4108,7 +4138,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -4166,7 +4196,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -4224,7 +4254,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="X65" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -4282,7 +4312,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -4340,7 +4370,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -4398,7 +4428,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -4456,7 +4486,7 @@
           <t>KLEVLEEV Anvar</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>130188</t>
         </is>
@@ -4514,7 +4544,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -4572,7 +4602,7 @@
           <t>HENDRICK Robert</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>43002</t>
         </is>
@@ -4630,7 +4660,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -4688,7 +4718,7 @@
           <t>BOBON Alexis</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>78745</t>
         </is>
@@ -4746,7 +4776,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -4804,7 +4834,7 @@
           <t>HANEDA Takuya</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="X75" t="inlineStr">
         <is>
           <t>36481</t>
         </is>
@@ -4862,7 +4892,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -4920,7 +4950,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -4978,7 +5008,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="X78" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -5036,7 +5066,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="X79" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -5094,7 +5124,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="X80" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -5152,7 +5182,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr">
+      <c r="X81" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -5210,7 +5240,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="X82" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -5480,7 +5510,7 @@
           <t>SATKOVA Gabriela</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
+      <c r="X87" t="inlineStr">
         <is>
           <t>68786</t>
         </is>
@@ -5538,7 +5568,7 @@
           <t>CORCORAN Madison</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="X88" t="inlineStr">
         <is>
           <t>106163</t>
         </is>
@@ -5596,7 +5626,7 @@
           <t>DUSKOVA Katerina</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr">
+      <c r="X89" t="inlineStr">
         <is>
           <t>51792</t>
         </is>
@@ -5654,7 +5684,7 @@
           <t>KUZNETSOVA Daria</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr">
+      <c r="X90" t="inlineStr">
         <is>
           <t>76780</t>
         </is>
@@ -5712,7 +5742,7 @@
           <t>SEPRENYI Sara Timea</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="X91" t="inlineStr">
         <is>
           <t>52211</t>
         </is>
@@ -5770,7 +5800,7 @@
           <t>KRYLOVA Kseniia</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="X92" t="inlineStr">
         <is>
           <t>60639</t>
         </is>
@@ -5828,7 +5858,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="X93" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -5886,7 +5916,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U94" t="inlineStr">
+      <c r="X94" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -5944,7 +5974,7 @@
           <t>PRIGENT Romane</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="X95" t="inlineStr">
         <is>
           <t>71968</t>
         </is>
@@ -6002,7 +6032,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="X96" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -6060,7 +6090,7 @@
           <t>OSCHMAUTZ Antonia</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr">
+      <c r="X97" t="inlineStr">
         <is>
           <t>68839</t>
         </is>
@@ -6118,7 +6148,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="X98" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -6176,7 +6206,7 @@
           <t>YAZAWA Aki</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="X99" t="inlineStr">
         <is>
           <t>36486</t>
         </is>
@@ -6234,7 +6264,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="X100" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -6292,7 +6322,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U101" t="inlineStr">
+      <c r="X101" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -6350,7 +6380,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="X102" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -6408,7 +6438,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="X103" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -6466,7 +6496,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="X104" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -6524,7 +6554,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
+      <c r="X105" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -6582,7 +6612,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="X106" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -6640,7 +6670,7 @@
           <t>FRIEDENSON Kaelin</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="X107" t="inlineStr">
         <is>
           <t>87397</t>
         </is>
@@ -6698,7 +6728,7 @@
           <t>JEVTIC Milos</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="X108" t="inlineStr">
         <is>
           <t>68832</t>
         </is>
@@ -6756,7 +6786,7 @@
           <t>RUDORFER Martin</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>83774</t>
         </is>
@@ -6814,7 +6844,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="X110" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -6872,7 +6902,7 @@
           <t>CURTIS Samuel</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="X111" t="inlineStr">
         <is>
           <t>36683</t>
         </is>
@@ -6930,7 +6960,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
+      <c r="X112" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -6988,7 +7018,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr">
+      <c r="X113" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -7046,7 +7076,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="X114" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -7104,7 +7134,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="X115" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -7162,7 +7192,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="X116" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -7220,7 +7250,7 @@
           <t>MARX Dimitri</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr">
+      <c r="X117" t="inlineStr">
         <is>
           <t>60326</t>
         </is>
@@ -7278,7 +7308,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="X118" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -7336,7 +7366,7 @@
           <t>KREJCI Jakub</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="X119" t="inlineStr">
         <is>
           <t>83510</t>
         </is>
@@ -7394,7 +7424,7 @@
           <t>ZIMA Tomas</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="X120" t="inlineStr">
         <is>
           <t>60019</t>
         </is>
@@ -7452,7 +7482,7 @@
           <t>HENE Simon</t>
         </is>
       </c>
-      <c r="U121" t="inlineStr">
+      <c r="X121" t="inlineStr">
         <is>
           <t>78750</t>
         </is>
@@ -7510,7 +7540,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="X122" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -7568,7 +7598,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="X123" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -7626,7 +7656,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="X124" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -7684,7 +7714,7 @@
           <t>DELASSUS Anatole</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr">
+      <c r="X125" t="inlineStr">
         <is>
           <t>84109</t>
         </is>
@@ -7742,7 +7772,7 @@
           <t>TSVIET Igor</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
+      <c r="X126" t="inlineStr">
         <is>
           <t>35527</t>
         </is>
@@ -7800,7 +7830,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr">
+      <c r="X127" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -7858,7 +7888,7 @@
           <t>KUDER MARUSIC Vid</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
+      <c r="X128" t="inlineStr">
         <is>
           <t>44342</t>
         </is>
@@ -7916,7 +7946,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U129" t="inlineStr">
+      <c r="X129" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -7974,7 +8004,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
+      <c r="X130" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -8032,7 +8062,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr">
+      <c r="X131" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -8090,7 +8120,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="X132" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -8148,7 +8178,7 @@
           <t>EIGEL Pavel</t>
         </is>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>35458</t>
         </is>
@@ -8206,7 +8236,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="X134" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -8264,7 +8294,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -8322,7 +8352,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="X136" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -8380,7 +8410,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr">
+      <c r="X137" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -8448,7 +8478,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
+      <c r="X138" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -8516,7 +8546,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="X139" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -8584,7 +8614,7 @@
           <t>OSCHMAUTZ Antonia</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="X140" t="inlineStr">
         <is>
           <t>68839</t>
         </is>
@@ -8652,7 +8682,7 @@
           <t>YAZAWA Aki</t>
         </is>
       </c>
-      <c r="U141" t="inlineStr">
+      <c r="X141" t="inlineStr">
         <is>
           <t>36486</t>
         </is>
@@ -8720,7 +8750,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="X142" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -8788,7 +8818,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="X143" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -8856,7 +8886,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="X144" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -8924,7 +8954,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr">
+      <c r="X145" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -8992,7 +9022,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="X146" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -9060,7 +9090,7 @@
           <t>PRIGENT Romane</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="X147" t="inlineStr">
         <is>
           <t>71968</t>
         </is>
@@ -9128,7 +9158,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr">
+      <c r="X148" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -9196,7 +9226,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr">
+      <c r="X149" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -9264,7 +9294,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
+      <c r="X150" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -9332,7 +9362,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr">
+      <c r="X151" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -9400,7 +9430,7 @@
           <t>KUDER MARUSIC Vid</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="X152" t="inlineStr">
         <is>
           <t>44342</t>
         </is>
@@ -9468,7 +9498,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
+      <c r="X153" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -9536,7 +9566,7 @@
           <t>KREJCI Jakub</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="X154" t="inlineStr">
         <is>
           <t>83510</t>
         </is>
@@ -9604,7 +9634,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="X155" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -9672,7 +9702,7 @@
           <t>HENE Simon</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="X156" t="inlineStr">
         <is>
           <t>78750</t>
         </is>
@@ -9740,7 +9770,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
+      <c r="X157" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -9803,7 +9833,7 @@
           <t>JAN STUPICA Neza</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="X158" t="inlineStr">
         <is>
           <t>105699</t>
         </is>
@@ -9866,7 +9896,7 @@
           <t>PRIGENT Romane</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="X159" t="inlineStr">
         <is>
           <t>71968</t>
         </is>
@@ -9929,7 +9959,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="X160" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -9992,7 +10022,7 @@
           <t>DUSKOVA Katerina</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr">
+      <c r="X161" t="inlineStr">
         <is>
           <t>51792</t>
         </is>
@@ -10055,7 +10085,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="X162" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -10118,7 +10148,7 @@
           <t>KUZNETSOVA Daria</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr">
+      <c r="X163" t="inlineStr">
         <is>
           <t>76780</t>
         </is>
@@ -10181,7 +10211,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr">
+      <c r="X164" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -10244,7 +10274,7 @@
           <t>FRIEDENSON Kaelin</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr">
+      <c r="X165" t="inlineStr">
         <is>
           <t>87397</t>
         </is>
@@ -10307,7 +10337,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
+      <c r="X166" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -10370,7 +10400,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="X167" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -10433,7 +10463,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="X168" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -10496,7 +10526,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
+      <c r="X169" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -10559,7 +10589,7 @@
           <t>TERCELJ Matic</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
+      <c r="X170" t="inlineStr">
         <is>
           <t>87126</t>
         </is>
@@ -10622,7 +10652,7 @@
           <t>KREJCI Jakub</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="X171" t="inlineStr">
         <is>
           <t>83510</t>
         </is>
@@ -10685,7 +10715,7 @@
           <t>SAVLI Erazem</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>72625</t>
         </is>
@@ -10748,7 +10778,7 @@
           <t>EIGEL Pavel</t>
         </is>
       </c>
-      <c r="U173" t="inlineStr">
+      <c r="X173" t="inlineStr">
         <is>
           <t>35458</t>
         </is>
@@ -10811,7 +10841,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="X174" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -10874,7 +10904,7 @@
           <t>RUDORFER Martin</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr">
+      <c r="X175" t="inlineStr">
         <is>
           <t>83774</t>
         </is>
@@ -10937,7 +10967,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U176" t="inlineStr">
+      <c r="X176" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -11000,7 +11030,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
+      <c r="X177" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -11063,7 +11093,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="X178" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -11126,7 +11156,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="X179" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -11189,7 +11219,7 @@
           <t>SAVLI Jakob</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="X180" t="inlineStr">
         <is>
           <t>96696</t>
         </is>
@@ -11252,7 +11282,7 @@
           <t>EIGEL Pavel</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr">
+      <c r="X181" t="inlineStr">
         <is>
           <t>35458</t>
         </is>
@@ -11315,7 +11345,7 @@
           <t>RUDORFER Martin</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
+      <c r="X182" t="inlineStr">
         <is>
           <t>83774</t>
         </is>
@@ -11378,7 +11408,7 @@
           <t>SAVLI Erazem</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="X183" t="inlineStr">
         <is>
           <t>72625</t>
         </is>
@@ -11441,7 +11471,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="X184" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -11504,7 +11534,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr">
+      <c r="X185" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -11567,7 +11597,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr">
+      <c r="X186" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -11630,7 +11660,7 @@
           <t>SAVLI Jakob</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>96696</t>
         </is>
@@ -11693,7 +11723,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="X188" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -11756,7 +11786,7 @@
           <t>FRIEDENSON Kaelin</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
+      <c r="X189" t="inlineStr">
         <is>
           <t>87397</t>
         </is>
@@ -11819,7 +11849,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr">
+      <c r="X190" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -11882,7 +11912,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="X191" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -11945,7 +11975,7 @@
           <t>TERCELJ Matic</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr">
+      <c r="X192" t="inlineStr">
         <is>
           <t>87126</t>
         </is>
@@ -12008,7 +12038,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
+      <c r="X193" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -12071,7 +12101,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -12134,7 +12164,7 @@
           <t>KREJCI Jakub</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="X195" t="inlineStr">
         <is>
           <t>83510</t>
         </is>
@@ -12197,7 +12227,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="X196" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -12260,7 +12290,7 @@
           <t>DUSKOVA Katerina</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr">
+      <c r="X197" t="inlineStr">
         <is>
           <t>51792</t>
         </is>
@@ -12323,7 +12353,7 @@
           <t>JAN STUPICA Neza</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="X198" t="inlineStr">
         <is>
           <t>105699</t>
         </is>
@@ -12386,7 +12416,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="X199" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -12449,7 +12479,7 @@
           <t>PRIGENT Romane</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="X200" t="inlineStr">
         <is>
           <t>71968</t>
         </is>
@@ -12512,6 +12542,11 @@
           <t>CORCORAN Michaela</t>
         </is>
       </c>
+      <c r="X201" t="inlineStr">
+        <is>
+          <t>106164</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -12570,7 +12605,7 @@
           <t>KUZNETSOVA Daria</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
+      <c r="X202" t="inlineStr">
         <is>
           <t>76780</t>
         </is>
@@ -12633,7 +12668,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U203" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -12696,7 +12731,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr">
+      <c r="X204" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -12759,7 +12794,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
+      <c r="X205" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -12822,7 +12857,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U206" t="inlineStr">
+      <c r="X206" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -12885,7 +12920,7 @@
           <t>RUDORFER Martin</t>
         </is>
       </c>
-      <c r="U207" t="inlineStr">
+      <c r="X207" t="inlineStr">
         <is>
           <t>83774</t>
         </is>
@@ -12948,7 +12983,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
+      <c r="X208" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -13011,7 +13046,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
+      <c r="X209" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -13074,7 +13109,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr">
+      <c r="X210" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -13137,7 +13172,7 @@
           <t>KREJCI Jakub</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
+      <c r="X211" t="inlineStr">
         <is>
           <t>83510</t>
         </is>
@@ -13200,7 +13235,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
+      <c r="X212" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -13273,7 +13308,7 @@
           <t>KUZNETSOVA Daria</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
+      <c r="X213" t="inlineStr">
         <is>
           <t>76780</t>
         </is>
@@ -13346,7 +13381,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
+      <c r="X214" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -13409,7 +13444,7 @@
           <t>PRIGENT Romane</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr">
+      <c r="X215" t="inlineStr">
         <is>
           <t>71968</t>
         </is>
@@ -13472,7 +13507,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
+      <c r="X216" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -13545,7 +13580,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr">
+      <c r="X217" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -13618,7 +13653,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
+      <c r="X218" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -13691,7 +13726,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U219" t="inlineStr">
+      <c r="X219" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -13764,7 +13799,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
+      <c r="X220" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -13981,7 +14016,7 @@
           <t>CORCORAN Michaela</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
+      <c r="X224" t="inlineStr">
         <is>
           <t>106164</t>
         </is>
@@ -14039,7 +14074,7 @@
           <t>SATO Ayano</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
+      <c r="X225" t="inlineStr">
         <is>
           <t>60374</t>
         </is>
@@ -14097,7 +14132,7 @@
           <t>KOZYREVA Anastasia</t>
         </is>
       </c>
-      <c r="U226" t="inlineStr">
+      <c r="X226" t="inlineStr">
         <is>
           <t>60640</t>
         </is>
@@ -14155,7 +14190,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
+      <c r="X227" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -14213,7 +14248,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U228" t="inlineStr">
+      <c r="X228" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -14271,7 +14306,7 @@
           <t>DOBROTVORSKA Viktoriia</t>
         </is>
       </c>
-      <c r="U229" t="inlineStr">
+      <c r="X229" t="inlineStr">
         <is>
           <t>35526</t>
         </is>
@@ -14329,7 +14364,7 @@
           <t>SATKOVA Gabriela</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
+      <c r="X230" t="inlineStr">
         <is>
           <t>68786</t>
         </is>
@@ -14387,7 +14422,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
+      <c r="X231" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -14445,7 +14480,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
+      <c r="X232" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -14503,7 +14538,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U233" t="inlineStr">
+      <c r="X233" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -14561,7 +14596,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
+      <c r="X234" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -14619,7 +14654,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
+      <c r="X235" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -14677,7 +14712,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
+      <c r="X236" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -14735,7 +14770,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr">
+      <c r="X237" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -14793,7 +14828,7 @@
           <t>KLEVLEEV Anvar</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr">
+      <c r="X238" t="inlineStr">
         <is>
           <t>130188</t>
         </is>
@@ -14851,7 +14886,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
+      <c r="X239" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -14909,7 +14944,7 @@
           <t>HENDRICK Robert</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
+      <c r="X240" t="inlineStr">
         <is>
           <t>43002</t>
         </is>
@@ -14967,7 +15002,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
+      <c r="X241" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -15025,7 +15060,7 @@
           <t>BOBON Alexis</t>
         </is>
       </c>
-      <c r="U242" t="inlineStr">
+      <c r="X242" t="inlineStr">
         <is>
           <t>78745</t>
         </is>
@@ -15083,7 +15118,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U243" t="inlineStr">
+      <c r="X243" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -15141,7 +15176,7 @@
           <t>HANEDA Takuya</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
+      <c r="X244" t="inlineStr">
         <is>
           <t>36481</t>
         </is>
@@ -15199,7 +15234,7 @@
           <t>BERNARDET Jules</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr">
+      <c r="X245" t="inlineStr">
         <is>
           <t>84123</t>
         </is>
@@ -15257,7 +15292,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr">
+      <c r="X246" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -15315,7 +15350,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
+      <c r="X247" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -15373,7 +15408,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
+      <c r="X248" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -15431,7 +15466,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U249" t="inlineStr">
+      <c r="X249" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -15489,7 +15524,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr">
+      <c r="X250" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -15547,7 +15582,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
+      <c r="X251" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -15605,7 +15640,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
+      <c r="X252" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -15673,7 +15708,7 @@
           <t>DOBROTVORSKA Viktoriia</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
+      <c r="X253" t="inlineStr">
         <is>
           <t>35526</t>
         </is>
@@ -15741,7 +15776,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U254" t="inlineStr">
+      <c r="X254" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -15809,7 +15844,7 @@
           <t>CORCORAN Michaela</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr">
+      <c r="X255" t="inlineStr">
         <is>
           <t>106164</t>
         </is>
@@ -15877,7 +15912,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
+      <c r="X256" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -15945,7 +15980,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr">
+      <c r="X257" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -16013,7 +16048,7 @@
           <t>LEIBFARTH Evy</t>
         </is>
       </c>
-      <c r="U258" t="inlineStr">
+      <c r="X258" t="inlineStr">
         <is>
           <t>83538</t>
         </is>
@@ -16081,7 +16116,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U259" t="inlineStr">
+      <c r="X259" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -16149,7 +16184,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U260" t="inlineStr">
+      <c r="X260" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -16217,7 +16252,7 @@
           <t>SATKOVA Gabriela</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
+      <c r="X261" t="inlineStr">
         <is>
           <t>68786</t>
         </is>
@@ -16285,7 +16320,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
+      <c r="X262" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -16353,7 +16388,7 @@
           <t>BERNARDET Jules</t>
         </is>
       </c>
-      <c r="U263" t="inlineStr">
+      <c r="X263" t="inlineStr">
         <is>
           <t>84123</t>
         </is>
@@ -16421,7 +16456,7 @@
           <t>KLEVLEEV Anvar</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
+      <c r="X264" t="inlineStr">
         <is>
           <t>130188</t>
         </is>
@@ -16542,7 +16577,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U266" t="inlineStr">
+      <c r="X266" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -16663,7 +16698,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U268" t="inlineStr">
+      <c r="X268" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -16837,7 +16872,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U271" t="inlineStr">
+      <c r="X271" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -17011,7 +17046,7 @@
           <t>BOBON Alexis</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
+      <c r="X274" t="inlineStr">
         <is>
           <t>78745</t>
         </is>
@@ -17132,7 +17167,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
+      <c r="X276" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -17200,7 +17235,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
+      <c r="X277" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -17268,7 +17303,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr">
+      <c r="X278" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -17336,7 +17371,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr">
+      <c r="X279" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -17805,11 +17840,16 @@
           <t>CORCORAN Michaela</t>
         </is>
       </c>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>106164</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -17822,14 +17862,9 @@
           <t>K1</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>Cross</t>
-        </is>
-      </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Time Trials</t>
+          <t>Forerunner</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -17844,28 +17879,23 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>13:49:30</t>
+          <t>14:21:00</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>AUT</t>
+          <t>SLO</t>
         </is>
       </c>
       <c r="J288" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K288" t="n">
         <v>257</v>
       </c>
       <c r="R288" t="inlineStr">
         <is>
-          <t>LEITNER Mario</t>
-        </is>
-      </c>
-      <c r="U288" t="inlineStr">
-        <is>
-          <t>35546</t>
+          <t>ZANOSKAR Zala</t>
         </is>
       </c>
     </row>
@@ -17885,14 +17915,9 @@
           <t>K1</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>Cross</t>
-        </is>
-      </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Time Trials</t>
+          <t>Forerunner</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -17907,35 +17932,30 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>13:50:15</t>
+          <t>14:22:00</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
         <is>
-          <t>CRO</t>
+          <t>SLO</t>
         </is>
       </c>
       <c r="J289" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="K289" t="n">
         <v>258</v>
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>KORPES Ren</t>
-        </is>
-      </c>
-      <c r="U289" t="inlineStr">
-        <is>
-          <t>39941</t>
+          <t>TOMINC Lan</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -17965,7 +17985,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>14:21:00</t>
+          <t>14:23:00</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -17974,14 +17994,14 @@
         </is>
       </c>
       <c r="J290" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K290" t="n">
         <v>259</v>
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>ZANOSKAR Zala</t>
+          <t>LOCNIKAR Jan</t>
         </is>
       </c>
     </row>
@@ -18018,7 +18038,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>14:22:00</t>
+          <t>14:26:00</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -18027,526 +18047,14 @@
         </is>
       </c>
       <c r="J291" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K291" t="n">
         <v>260</v>
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>TOMINC Lan</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>Forerunner</t>
-        </is>
-      </c>
-      <c r="F292" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G292" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H292" t="inlineStr">
-        <is>
-          <t>14:23:00</t>
-        </is>
-      </c>
-      <c r="I292" t="inlineStr">
-        <is>
-          <t>SLO</t>
-        </is>
-      </c>
-      <c r="J292" t="n">
-        <v>5</v>
-      </c>
-      <c r="K292" t="n">
-        <v>261</v>
-      </c>
-      <c r="R292" t="inlineStr">
-        <is>
-          <t>LOCNIKAR Jan</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>Forerunner</t>
-        </is>
-      </c>
-      <c r="F293" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G293" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>14:26:00</t>
-        </is>
-      </c>
-      <c r="I293" t="inlineStr">
-        <is>
-          <t>SLO</t>
-        </is>
-      </c>
-      <c r="J293" t="n">
-        <v>7</v>
-      </c>
-      <c r="K293" t="n">
-        <v>262</v>
-      </c>
-      <c r="R293" t="inlineStr">
-        <is>
           <t>POLENCIC Nejc</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C294" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F294" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G294" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H294" t="inlineStr">
-        <is>
-          <t>14:45:00</t>
-        </is>
-      </c>
-      <c r="I294" t="inlineStr">
-        <is>
-          <t>SLO</t>
-        </is>
-      </c>
-      <c r="J294" t="n">
-        <v>18</v>
-      </c>
-      <c r="K294" t="n">
-        <v>263</v>
-      </c>
-      <c r="R294" t="inlineStr">
-        <is>
-          <t>HOCEVAR Eva Alina</t>
-        </is>
-      </c>
-      <c r="U294" t="inlineStr">
-        <is>
-          <t>75533</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C295" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F295" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G295" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H295" t="inlineStr">
-        <is>
-          <t>14:53:00</t>
-        </is>
-      </c>
-      <c r="I295" t="inlineStr">
-        <is>
-          <t>AUT</t>
-        </is>
-      </c>
-      <c r="J295" t="n">
-        <v>10</v>
-      </c>
-      <c r="K295" t="n">
-        <v>264</v>
-      </c>
-      <c r="R295" t="inlineStr">
-        <is>
-          <t>WERATSCHNIG Nina</t>
-        </is>
-      </c>
-      <c r="U295" t="inlineStr">
-        <is>
-          <t>41614</t>
-        </is>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C296" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F296" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G296" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H296" t="inlineStr">
-        <is>
-          <t>15:02:00</t>
-        </is>
-      </c>
-      <c r="I296" t="inlineStr">
-        <is>
-          <t>AUT</t>
-        </is>
-      </c>
-      <c r="J296" t="n">
-        <v>1</v>
-      </c>
-      <c r="K296" t="n">
-        <v>265</v>
-      </c>
-      <c r="R296" t="inlineStr">
-        <is>
-          <t>KUHNLE Corinna</t>
-        </is>
-      </c>
-      <c r="U296" t="inlineStr">
-        <is>
-          <t>35282</t>
-        </is>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C297" t="inlineStr">
-        <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="E297" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F297" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G297" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H297" t="inlineStr">
-        <is>
-          <t>15:21:00</t>
-        </is>
-      </c>
-      <c r="I297" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="J297" t="n">
-        <v>17</v>
-      </c>
-      <c r="K297" t="n">
-        <v>266</v>
-      </c>
-      <c r="R297" t="inlineStr">
-        <is>
-          <t>HENE Simon</t>
-        </is>
-      </c>
-      <c r="U297" t="inlineStr">
-        <is>
-          <t>78750</t>
-        </is>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C298" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="E298" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F298" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G298" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H298" t="inlineStr">
-        <is>
-          <t>15:45:00</t>
-        </is>
-      </c>
-      <c r="I298" t="inlineStr">
-        <is>
-          <t>SLO</t>
-        </is>
-      </c>
-      <c r="J298" t="n">
-        <v>16</v>
-      </c>
-      <c r="K298" t="n">
-        <v>267</v>
-      </c>
-      <c r="R298" t="inlineStr">
-        <is>
-          <t>HOCEVAR Eva Alina</t>
-        </is>
-      </c>
-      <c r="U298" t="inlineStr">
-        <is>
-          <t>75533</t>
-        </is>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="inlineStr">
-        <is>
-          <t>W</t>
-        </is>
-      </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="E299" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F299" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G299" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H299" t="inlineStr">
-        <is>
-          <t>15:59:00</t>
-        </is>
-      </c>
-      <c r="I299" t="inlineStr">
-        <is>
-          <t>AUT</t>
-        </is>
-      </c>
-      <c r="J299" t="n">
-        <v>2</v>
-      </c>
-      <c r="K299" t="n">
-        <v>268</v>
-      </c>
-      <c r="R299" t="inlineStr">
-        <is>
-          <t>WERATSCHNIG Nadine</t>
-        </is>
-      </c>
-      <c r="U299" t="inlineStr">
-        <is>
-          <t>41613</t>
-        </is>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>SENIOR</t>
-        </is>
-      </c>
-      <c r="C300" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="E300" t="inlineStr">
-        <is>
-          <t>Heats</t>
-        </is>
-      </c>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G300" t="inlineStr">
-        <is>
-          <t>2020-10-18</t>
-        </is>
-      </c>
-      <c r="H300" t="inlineStr">
-        <is>
-          <t>16:12:00</t>
-        </is>
-      </c>
-      <c r="I300" t="inlineStr">
-        <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="J300" t="n">
-        <v>8</v>
-      </c>
-      <c r="K300" t="n">
-        <v>269</v>
-      </c>
-      <c r="R300" t="inlineStr">
-        <is>
-          <t>BERNARDET Jules</t>
-        </is>
-      </c>
-      <c r="U300" t="inlineStr">
-        <is>
-          <t>84123</t>
         </is>
       </c>
     </row>

</xml_diff>